<commit_message>
Fix critical review flaws across dashboard, skills, and docs
</commit_message>
<xml_diff>
--- a/excel/JobHunter_Pipeline.xlsx
+++ b/excel/JobHunter_Pipeline.xlsx
@@ -20,8 +20,30 @@
 </workbook>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>JobHunter OS</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Add rows below, or ask your agent to 'find me jobs' / 'find me jobs in Excel'.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="24">
   <si>
     <t xml:space="preserve">JobHunter OS — Pipeline Dashboard</t>
   </si>
@@ -93,99 +115,6 @@
   </si>
   <si>
     <t xml:space="preserve">Job URL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Northwind Retail</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operations Manager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://example.com/1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vertex Logistics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Supply Chain Lead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://example.com/2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bright Harbor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Category Manager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://example.com/3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acme Freight</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://example.com/4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Globex Corp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Business Ops Lead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-07-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://example.com/5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initech</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Procurement Manager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://example.com/6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Umbrella Retail</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ops Director</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://example.com/7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stellar Group</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://example.com/8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wayne Logistics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://example.com/9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sample Co</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ops Coordinator</t>
   </si>
 </sst>
 </file>
@@ -195,7 +124,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -299,6 +228,11 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -476,7 +410,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="25">
+  <dxfs count="10">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -488,126 +422,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD7F4E7"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEDEDF0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFBDCE6"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEAD2"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF2CB67D"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF6F7287"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB25E00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE53170"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE6E6E9"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFBE2DC"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF1E8A5F"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4B4D60"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB4402E"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC21C5C"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -903,22 +718,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>4</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -926,11 +741,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="28192804"/>
-        <c:axId val="3803775"/>
+        <c:axId val="63824090"/>
+        <c:axId val="69385287"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="28192804"/>
+        <c:axId val="63824090"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -963,7 +778,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="3803775"/>
+        <c:crossAx val="69385287"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -971,7 +786,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="3803775"/>
+        <c:axId val="69385287"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1047,7 +862,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="28192804"/>
+        <c:crossAx val="63824090"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1347,16 +1162,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>5</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1913,8 +1728,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PipelineTable" displayName="PipelineTable" ref="A1:G11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:G11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PipelineTable" displayName="PipelineTable" ref="A1:G1" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:G1"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Company"/>
     <tableColumn id="2" name="Role"/>
@@ -2150,19 +1965,19 @@
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="7" t="n">
         <f aca="false">COUNTA(Pipeline!A2:A500)</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C7" s="7" t="n">
         <f aca="false">COUNTIF(Pipeline!E2:E500,"Applied")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D7" s="7" t="n">
         <f aca="false">COUNTIF(Pipeline!E2:E500,"Interviewing")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" s="7" t="n">
         <f aca="false">COUNTIF(Pipeline!E2:E500,"Offer")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2199,14 +2014,14 @@
       </c>
       <c r="C14" s="10" t="n">
         <f aca="false">COUNTIFS(Pipeline!C2:C500,"&gt;=80")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>12</v>
       </c>
       <c r="F14" s="10" t="n">
         <f aca="false">COUNTIF(Pipeline!E2:E500,"Scouted")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2215,14 +2030,14 @@
       </c>
       <c r="C15" s="10" t="n">
         <f aca="false">COUNTIFS(Pipeline!C2:C500,"&gt;=70",Pipeline!C2:C500,"&lt;80")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>14</v>
       </c>
       <c r="F15" s="10" t="n">
         <f aca="false">COUNTIF(Pipeline!E2:E500,"CV Ready")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2231,14 +2046,14 @@
       </c>
       <c r="C16" s="10" t="n">
         <f aca="false">COUNTIFS(Pipeline!C2:C500,"&gt;=60",Pipeline!C2:C500,"&lt;70")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>3</v>
       </c>
       <c r="F16" s="10" t="n">
         <f aca="false">COUNTIF(Pipeline!E2:E500,"Applied")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2247,14 +2062,14 @@
       </c>
       <c r="C17" s="10" t="n">
         <f aca="false">COUNTIFS(Pipeline!C2:C500,"&lt;60",Pipeline!C2:C500,"&lt;&gt;")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F17" s="10" t="n">
         <f aca="false">COUNTIF(Pipeline!E2:E500,"Interviewing")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2263,7 +2078,7 @@
       </c>
       <c r="F18" s="10" t="n">
         <f aca="false">COUNTIF(Pipeline!E2:E500,"Offer")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2272,7 +2087,7 @@
       </c>
       <c r="F19" s="10" t="n">
         <f aca="false">COUNTIF(Pipeline!E2:E500,"Rejected")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2302,7 +2117,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="22"/>
@@ -2335,264 +2150,38 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" s="10" t="n">
-        <v>88</v>
-      </c>
-      <c r="D2" s="10" t="str">
-        <f aca="false">IF(C2="","",IF(C2&gt;=80,"HOT",IF(C2&gt;=70,"Strong",IF(C2&gt;=60,"Consider","Low"))))</f>
-        <v>HOT</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C3" s="10" t="n">
-        <v>74</v>
-      </c>
-      <c r="D3" s="10" t="str">
-        <f aca="false">IF(C3="","",IF(C3&gt;=80,"HOT",IF(C3&gt;=70,"Strong",IF(C3&gt;=60,"Consider","Low"))))</f>
-        <v>Strong</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" s="10" t="n">
-        <v>61</v>
-      </c>
-      <c r="D4" s="10" t="str">
-        <f aca="false">IF(C4="","",IF(C4&gt;=80,"HOT",IF(C4&gt;=70,"Strong",IF(C4&gt;=60,"Consider","Low"))))</f>
-        <v>Consider</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" s="10" t="n">
-        <v>91</v>
-      </c>
-      <c r="D5" s="10" t="str">
-        <f aca="false">IF(C5="","",IF(C5&gt;=80,"HOT",IF(C5&gt;=70,"Strong",IF(C5&gt;=60,"Consider","Low"))))</f>
-        <v>HOT</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C6" s="10" t="n">
-        <v>83</v>
-      </c>
-      <c r="D6" s="10" t="str">
-        <f aca="false">IF(C6="","",IF(C6&gt;=80,"HOT",IF(C6&gt;=70,"Strong",IF(C6&gt;=60,"Consider","Low"))))</f>
-        <v>HOT</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" s="10" t="n">
-        <v>69</v>
-      </c>
-      <c r="D7" s="10" t="str">
-        <f aca="false">IF(C7="","",IF(C7&gt;=80,"HOT",IF(C7&gt;=70,"Strong",IF(C7&gt;=60,"Consider","Low"))))</f>
-        <v>Consider</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="C8" s="10" t="n">
-        <v>85</v>
-      </c>
-      <c r="D8" s="10" t="str">
-        <f aca="false">IF(C8="","",IF(C8&gt;=80,"HOT",IF(C8&gt;=70,"Strong",IF(C8&gt;=60,"Consider","Low"))))</f>
-        <v>HOT</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="10" t="n">
-        <v>90</v>
-      </c>
-      <c r="D9" s="10" t="str">
-        <f aca="false">IF(C9="","",IF(C9&gt;=80,"HOT",IF(C9&gt;=70,"Strong",IF(C9&gt;=60,"Consider","Low"))))</f>
-        <v>HOT</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" s="10" t="n">
-        <v>55</v>
-      </c>
-      <c r="D10" s="10" t="str">
-        <f aca="false">IF(C10="","",IF(C10&gt;=80,"HOT",IF(C10&gt;=70,"Strong",IF(C10&gt;=60,"Consider","Low"))))</f>
-        <v>Low</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10" t="str">
-        <f aca="false">IF(C11="","",IF(C11&gt;=80,"HOT",IF(C11&gt;=70,"Strong",IF(C11&gt;=60,"Consider","Low"))))</f>
-        <v/>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10"/>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:D11">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+  <conditionalFormatting sqref="D2:D500">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>"HOT"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>"Strong"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>"Consider"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>"Low"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E11">
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
+  <conditionalFormatting sqref="E2:E500">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>"Scouted"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"CV Ready"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>"Applied"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="22">
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"Interviewing"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="23">
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Offer"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="24">
+    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>"Rejected"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2603,8 +2192,9 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <legacyDrawing r:id="rId2"/>
   <tableParts>
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>